<commit_message>
Add G10 rate sensitivity to Brent; fix secondary axis position
The construction chart had its second value axis at axPos=l, so both scales
stacked on the left rather than one moving to the right. The category axis
had the same defect. Both now set explicitly.

New chart 6: the slope of each G10 10y, in basis points, on the weekly per
cent change in Brent, Friday to Friday since February 2026. Seven markets
only - no free daily 10y was reachable for Canada, Switzerland or New
Zealand, and they are left out rather than proxied.

The estimates move materially with the sampling weekday, so the ranking is
the readable part, not the level. R squared per market is on the sheet.
</commit_message>
<xml_diff>
--- a/Market_Charts.xlsx
+++ b/Market_Charts.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuing" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bubbles" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Construction" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RateOilBeta" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -344,7 +345,7 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <numFmt formatCode="mmm-yy" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -707,7 +708,7 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
@@ -1040,7 +1041,7 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
@@ -1155,7 +1156,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="r"/>
         <title>
           <tx>
             <rich>
@@ -1496,7 +1498,7 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
@@ -1795,7 +1797,7 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <numFmt formatCode="mmm-yy" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -1911,7 +1913,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="r"/>
         <title>
           <tx>
             <rich>
@@ -1995,6 +1998,201 @@
         </a:p>
       </txPr>
     </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>10y rate sensitivity to Brent</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>bps per % Brent</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="DB0011"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'RateOilBeta'!$A$7:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'RateOilBeta'!$B$7:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="0.00"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="900" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="3175">
+              <a:solidFill>
+                <a:srgbClr val="D0CECE"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -2114,6 +2312,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>119</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7560000" cy="3780000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2412,7 +2632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2501,115 +2721,135 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6  Rate-oil beta</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>How far each G10 10y moves for a one per cent move in Brent, on weekly changes since February 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Yahoo Finance</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>ACWI, IEF and ^SPGSCI daily closes. The ETF series use the adjusted close, so distributions are reinvested; the S&amp;P GSCI is a spot index.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>FRED</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>ICSA, CCSA, UNRATE and DGS10.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>US Census Bureau</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>C30 value of construction put in place, private, seasonally adjusted. The data centre series is not carried on FRED and comes from the Census file directly.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>FRED</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>WPUSI012011, PPI construction materials, used to deflate.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>◆  Rebasing divides each series by its own first close and multiplies by 100, so every line starts together and the chart reads as relative performance.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>◆  The cross-asset spine is every weekday, with the previous close carried through a market holiday.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>◆  The dashed line on chart 2 is the 2023-25 average across all weeks, computed live on the Claims sheet. It is a reference for reading 2026 against, not a threshold with any meaning of its own.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>◆  Chart 4 measures each episode from its own start date. Yields rose in four of the six and fell in two. The current episode runs from 26 June 2025 and is not complete.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>◆  Chart 5 is nominal, which is how this is usually drawn. Columns E-G of the Construction sheet repeat it in January 2024 prices. Data centres sit on the right-hand scale.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>◆  Chart 6 is a plain least-squares slope of the weekly change in each 10y, in basis points, on the weekly per cent change in Brent, Friday to Friday. The estimates move materially with the sampling day - Britain ranges from 0.83 to 1.11 across Monday, Wednesday and Friday sampling - so read the ranking, not the level. R squared per market is on the RateOilBeta sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Built 08 August 2026. Rebuilt from primary sources rather than reproduced from third-party research.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A21:F21"/>
   </mergeCells>
@@ -39637,4 +39877,245 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>10y rate sensitivity to Brent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Basis points per one per cent move in Brent, from weekly Friday-to-Friday changes since February 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Sensitivity (bps per % Brent)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>R squared</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GB 10y</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>1.0581</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>0.5942</v>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>riksbank</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>GBGVB10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AU 10y</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>0.6802</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>rba</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>FCMYGBAG10D</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SE 10y</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>0.4589</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>riksbank</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>SEGVB10YC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>EU 10y</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.4735</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>riksbank</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>DEGVB10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>US 10y</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>fred</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>DGS10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>NO 10y</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>0.5847</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>0.3512</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>riksbank</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>NOGVB10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>JP 10y</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>0.2036</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>0.06569999999999999</v>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>riksbank</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>JPGVB10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Canada, Switzerland and New Zealand are absent because no free daily source for their 10y was reachable: the Bank of Canada benchmark series has stopped returning observations, the SNB bond cube is monthly and ends July 2025, and the RBNZ blocks automated requests. They are left out rather than proxied.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A16:F16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>